<commit_message>
Cutover rehearsal, go/no-go with a named fallback, and six dry-run checks across the series
</commit_message>
<xml_diff>
--- a/guides/data-migration-stages/toolkit/Data-Migration-Toolkit-TEMPLATE.xlsx
+++ b/guides/data-migration-stages/toolkit/Data-Migration-Toolkit-TEMPLATE.xlsx
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="F2" s="22" t="n">
-        <v>46101</v>
+        <v>46094</v>
       </c>
       <c r="G2" s="21" t="inlineStr">
         <is>
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="B13" s="10">
-        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$67,"1.*",'Migration Plan'!$F$2:$F$67,"Done")/COUNTIF('Migration Plan'!$B$2:$B$67,"1.*"),0)</f>
+        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$69,"1.*",'Migration Plan'!$F$2:$F$69,"Done")/COUNTIF('Migration Plan'!$B$2:$B$69,"1.*"),0)</f>
         <v/>
       </c>
     </row>
@@ -1070,7 +1070,7 @@
         </is>
       </c>
       <c r="B14" s="10">
-        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$67,"2.*",'Migration Plan'!$F$2:$F$67,"Done")/COUNTIF('Migration Plan'!$B$2:$B$67,"2.*"),0)</f>
+        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$69,"2.*",'Migration Plan'!$F$2:$F$69,"Done")/COUNTIF('Migration Plan'!$B$2:$B$69,"2.*"),0)</f>
         <v/>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
         </is>
       </c>
       <c r="B15" s="10">
-        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$67,"3.*",'Migration Plan'!$F$2:$F$67,"Done")/COUNTIF('Migration Plan'!$B$2:$B$67,"3.*"),0)</f>
+        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$69,"3.*",'Migration Plan'!$F$2:$F$69,"Done")/COUNTIF('Migration Plan'!$B$2:$B$69,"3.*"),0)</f>
         <v/>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="B16" s="10">
-        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$67,"4.*",'Migration Plan'!$F$2:$F$67,"Done")/COUNTIF('Migration Plan'!$B$2:$B$67,"4.*"),0)</f>
+        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$69,"4.*",'Migration Plan'!$F$2:$F$69,"Done")/COUNTIF('Migration Plan'!$B$2:$B$69,"4.*"),0)</f>
         <v/>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="B17" s="10">
-        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$67,"5.*",'Migration Plan'!$F$2:$F$67,"Done")/COUNTIF('Migration Plan'!$B$2:$B$67,"5.*"),0)</f>
+        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$69,"5.*",'Migration Plan'!$F$2:$F$69,"Done")/COUNTIF('Migration Plan'!$B$2:$B$69,"5.*"),0)</f>
         <v/>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="B18" s="10">
-        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$67,"6.*",'Migration Plan'!$F$2:$F$67,"Done")/COUNTIF('Migration Plan'!$B$2:$B$67,"6.*"),0)</f>
+        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$69,"6.*",'Migration Plan'!$F$2:$F$69,"Done")/COUNTIF('Migration Plan'!$B$2:$B$69,"6.*"),0)</f>
         <v/>
       </c>
     </row>
@@ -1125,7 +1125,7 @@
         </is>
       </c>
       <c r="B19" s="10">
-        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$67,"7.*",'Migration Plan'!$F$2:$F$67,"Done")/COUNTIF('Migration Plan'!$B$2:$B$67,"7.*"),0)</f>
+        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$69,"7.*",'Migration Plan'!$F$2:$F$69,"Done")/COUNTIF('Migration Plan'!$B$2:$B$69,"7.*"),0)</f>
         <v/>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
         </is>
       </c>
       <c r="B20" s="10">
-        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$67,"8.*",'Migration Plan'!$F$2:$F$67,"Done")/COUNTIF('Migration Plan'!$B$2:$B$67,"8.*"),0)</f>
+        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$69,"8.*",'Migration Plan'!$F$2:$F$69,"Done")/COUNTIF('Migration Plan'!$B$2:$B$69,"8.*"),0)</f>
         <v/>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="B21" s="10">
-        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$67,"DD.*",'Migration Plan'!$F$2:$F$67,"Done")/COUNTIF('Migration Plan'!$B$2:$B$67,"DD.*"),0)</f>
+        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$69,"DD.*",'Migration Plan'!$F$2:$F$69,"Done")/COUNTIF('Migration Plan'!$B$2:$B$69,"DD.*"),0)</f>
         <v/>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
         </is>
       </c>
       <c r="B22" s="10">
-        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$67,"BF.*",'Migration Plan'!$F$2:$F$67,"Done")/COUNTIF('Migration Plan'!$B$2:$B$67,"BF.*"),0)</f>
+        <f>IFERROR(COUNTIFS('Migration Plan'!$B$2:$B$69,"BF.*",'Migration Plan'!$F$2:$F$69,"Done")/COUNTIF('Migration Plan'!$B$2:$B$69,"BF.*"),0)</f>
         <v/>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="B23" s="12">
-        <f>IFERROR(COUNTIF('Migration Plan'!$F$2:$F$67,"Done")/COUNTA('Migration Plan'!$F$2:$F$67),0)</f>
+        <f>IFERROR(COUNTIF('Migration Plan'!$F$2:$F$69,"Done")/COUNTA('Migration Plan'!$F$2:$F$69),0)</f>
         <v/>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N67"/>
+  <dimension ref="A1:N69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="C33" s="16" t="inlineStr">
         <is>
-          <t>Run the four checks</t>
+          <t>Run the six checks</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -2779,14 +2779,14 @@
       <c r="H33" s="16" t="n"/>
       <c r="I33" s="16" t="n"/>
       <c r="J33" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K33" s="16" t="n">
         <v>26</v>
       </c>
       <c r="L33" s="16" t="inlineStr">
         <is>
-          <t>Counts, control totals, links, spot fidelity</t>
+          <t>Counts, control totals, links, spot fidelity, processability, integration</t>
         </is>
       </c>
       <c r="M33" s="16" t="inlineStr">
@@ -3319,7 +3319,7 @@
       </c>
       <c r="C45" s="16" t="inlineStr">
         <is>
-          <t>Take the final delta export</t>
+          <t>Full cutover rehearsal, timed against the freeze window</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="E45" s="16" t="inlineStr">
         <is>
-          <t>Client IT</t>
+          <t>Migration Lead</t>
         </is>
       </c>
       <c r="F45" s="16" t="inlineStr">
@@ -3343,14 +3343,14 @@
       <c r="H45" s="16" t="n"/>
       <c r="I45" s="16" t="n"/>
       <c r="J45" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K45" s="16" t="n">
         <v>36</v>
       </c>
       <c r="L45" s="16" t="inlineStr">
         <is>
-          <t>Everything added since the initial export</t>
+          <t>The whole sequence run end to end, clock running. Proves it fits.</t>
         </is>
       </c>
       <c r="M45" s="16" t="inlineStr">
@@ -3371,7 +3371,7 @@
       </c>
       <c r="C46" s="16" t="inlineStr">
         <is>
-          <t>Cutover, in order</t>
+          <t>Take the final delta export</t>
         </is>
       </c>
       <c r="D46" s="16" t="inlineStr">
@@ -3381,7 +3381,7 @@
       </c>
       <c r="E46" s="16" t="inlineStr">
         <is>
-          <t>Migration Lead</t>
+          <t>Client IT</t>
         </is>
       </c>
       <c r="F46" s="16" t="inlineStr">
@@ -3395,14 +3395,14 @@
       <c r="H46" s="16" t="n"/>
       <c r="I46" s="16" t="n"/>
       <c r="J46" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K46" s="16" t="n">
         <v>37</v>
       </c>
       <c r="L46" s="16" t="inlineStr">
         <is>
-          <t>Records, then documents, then links</t>
+          <t>Everything added since the initial export</t>
         </is>
       </c>
       <c r="M46" s="16" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="C47" s="16" t="inlineStr">
         <is>
-          <t>Bridge import</t>
+          <t>Go / no-go decision, with the fallback position named</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="E47" s="16" t="inlineStr">
         <is>
-          <t>Migration Lead</t>
+          <t>Client PM</t>
         </is>
       </c>
       <c r="F47" s="16" t="inlineStr">
@@ -3447,14 +3447,14 @@
       <c r="H47" s="16" t="n"/>
       <c r="I47" s="16" t="n"/>
       <c r="J47" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K47" s="16" t="n">
         <v>38</v>
       </c>
       <c r="L47" s="16" t="inlineStr">
         <is>
-          <t>The gap closed, not left for later</t>
+          <t>Who decides, on what evidence, and what happens if it is no</t>
         </is>
       </c>
       <c r="M47" s="16" t="inlineStr">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="C48" s="16" t="inlineStr">
         <is>
-          <t>Post-load reconciliation</t>
+          <t>Cutover, in order</t>
         </is>
       </c>
       <c r="D48" s="16" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="L48" s="16" t="inlineStr">
         <is>
-          <t>The same checks as the dry run, on production</t>
+          <t>Records, then documents, then links</t>
         </is>
       </c>
       <c r="M48" s="16" t="inlineStr">
@@ -3517,182 +3517,184 @@
       <c r="N48" s="16" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="18" t="n">
+      <c r="A49" s="16" t="n">
         <v>41</v>
       </c>
-      <c r="B49" s="18" t="inlineStr">
+      <c r="B49" s="16" t="inlineStr">
         <is>
           <t>7.6</t>
         </is>
       </c>
-      <c r="C49" s="19" t="inlineStr">
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>Bridge import</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>Stage 7 — Freeze, Cutover and Bridge</t>
+        </is>
+      </c>
+      <c r="E49" s="16" t="inlineStr">
+        <is>
+          <t>Migration Lead</t>
+        </is>
+      </c>
+      <c r="F49" s="16" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G49" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="16" t="n"/>
+      <c r="I49" s="16" t="n"/>
+      <c r="J49" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="K49" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="L49" s="16" t="inlineStr">
+        <is>
+          <t>The gap closed, not left for later</t>
+        </is>
+      </c>
+      <c r="M49" s="16" t="inlineStr">
+        <is>
+          <t>migration-cutover</t>
+        </is>
+      </c>
+      <c r="N49" s="16" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="n">
+        <v>42</v>
+      </c>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>7.7</t>
+        </is>
+      </c>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>Post-load reconciliation</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>Stage 7 — Freeze, Cutover and Bridge</t>
+        </is>
+      </c>
+      <c r="E50" s="16" t="inlineStr">
+        <is>
+          <t>Migration Lead</t>
+        </is>
+      </c>
+      <c r="F50" s="16" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G50" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="16" t="n"/>
+      <c r="I50" s="16" t="n"/>
+      <c r="J50" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="K50" s="16" t="n">
+        <v>41</v>
+      </c>
+      <c r="L50" s="16" t="inlineStr">
+        <is>
+          <t>The same six checks as the dry run, on production</t>
+        </is>
+      </c>
+      <c r="M50" s="16" t="inlineStr">
+        <is>
+          <t>migration-cutover</t>
+        </is>
+      </c>
+      <c r="N50" s="16" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="18" t="n">
+        <v>43</v>
+      </c>
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>7.8</t>
+        </is>
+      </c>
+      <c r="C51" s="19" t="inlineStr">
         <is>
           <t>GATE — go-live accepted</t>
         </is>
       </c>
-      <c r="D49" s="18" t="inlineStr">
+      <c r="D51" s="18" t="inlineStr">
         <is>
           <t>Stage 7 — Freeze, Cutover and Bridge</t>
         </is>
       </c>
-      <c r="E49" s="18" t="inlineStr">
+      <c r="E51" s="18" t="inlineStr">
         <is>
           <t>Client PM</t>
         </is>
       </c>
-      <c r="F49" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G49" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="18" t="n"/>
-      <c r="I49" s="18" t="n"/>
-      <c r="J49" s="18" t="n">
+      <c r="F51" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G51" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="18" t="n"/>
+      <c r="I51" s="18" t="n"/>
+      <c r="J51" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="K49" s="18" t="n">
-        <v>40</v>
-      </c>
-      <c r="L49" s="18" t="inlineStr">
+      <c r="K51" s="18" t="n">
+        <v>42</v>
+      </c>
+      <c r="L51" s="18" t="inlineStr">
         <is>
           <t>Numbers match, client accepts, together</t>
         </is>
       </c>
-      <c r="M49" s="18" t="inlineStr">
+      <c r="M51" s="18" t="inlineStr">
         <is>
           <t>migration-cutover</t>
         </is>
       </c>
-      <c r="N49" s="18" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="15" t="inlineStr"/>
-      <c r="B50" s="15" t="inlineStr">
+      <c r="N51" s="18" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="15" t="inlineStr"/>
+      <c r="B52" s="15" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="C50" s="15" t="inlineStr">
+      <c r="C52" s="15" t="inlineStr">
         <is>
           <t>Stage 8 — Hypercare and Close</t>
         </is>
       </c>
-      <c r="D50" s="15" t="inlineStr"/>
-      <c r="E50" s="15" t="inlineStr"/>
-      <c r="F50" s="15" t="inlineStr"/>
-      <c r="G50" s="15" t="inlineStr"/>
-      <c r="H50" s="15" t="inlineStr"/>
-      <c r="I50" s="15" t="inlineStr"/>
-      <c r="J50" s="15" t="inlineStr"/>
-      <c r="K50" s="15" t="inlineStr"/>
-      <c r="L50" s="15" t="inlineStr"/>
-      <c r="M50" s="15" t="inlineStr"/>
-      <c r="N50" s="15" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="16" t="n">
-        <v>42</v>
-      </c>
-      <c r="B51" s="16" t="inlineStr">
-        <is>
-          <t>8.1</t>
-        </is>
-      </c>
-      <c r="C51" s="16" t="inlineStr">
-        <is>
-          <t>Agree the hypercare window before you need it</t>
-        </is>
-      </c>
-      <c r="D51" s="16" t="inlineStr">
-        <is>
-          <t>Stage 8 — Hypercare and Close</t>
-        </is>
-      </c>
-      <c r="E51" s="16" t="inlineStr">
-        <is>
-          <t>Client PM</t>
-        </is>
-      </c>
-      <c r="F51" s="16" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G51" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H51" s="16" t="n"/>
-      <c r="I51" s="16" t="n"/>
-      <c r="J51" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="K51" s="16" t="inlineStr"/>
-      <c r="L51" s="16" t="inlineStr">
-        <is>
-          <t>Length and route agreed in advance</t>
-        </is>
-      </c>
-      <c r="M51" s="16" t="inlineStr">
-        <is>
-          <t>migration-hypercare</t>
-        </is>
-      </c>
-      <c r="N51" s="16" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="16" t="n">
-        <v>43</v>
-      </c>
-      <c r="B52" s="16" t="inlineStr">
-        <is>
-          <t>8.2</t>
-        </is>
-      </c>
-      <c r="C52" s="16" t="inlineStr">
-        <is>
-          <t>Log and resolve what surfaces</t>
-        </is>
-      </c>
-      <c r="D52" s="16" t="inlineStr">
-        <is>
-          <t>Stage 8 — Hypercare and Close</t>
-        </is>
-      </c>
-      <c r="E52" s="16" t="inlineStr">
-        <is>
-          <t>Migration Lead</t>
-        </is>
-      </c>
-      <c r="F52" s="16" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G52" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H52" s="16" t="n"/>
-      <c r="I52" s="16" t="n"/>
-      <c r="J52" s="16" t="n">
-        <v>15</v>
-      </c>
-      <c r="K52" s="16" t="n">
-        <v>42</v>
-      </c>
-      <c r="L52" s="16" t="inlineStr">
-        <is>
-          <t>The long tail, tracked not absorbed</t>
-        </is>
-      </c>
-      <c r="M52" s="16" t="inlineStr">
-        <is>
-          <t>migration-hypercare</t>
-        </is>
-      </c>
-      <c r="N52" s="16" t="inlineStr"/>
+      <c r="D52" s="15" t="inlineStr"/>
+      <c r="E52" s="15" t="inlineStr"/>
+      <c r="F52" s="15" t="inlineStr"/>
+      <c r="G52" s="15" t="inlineStr"/>
+      <c r="H52" s="15" t="inlineStr"/>
+      <c r="I52" s="15" t="inlineStr"/>
+      <c r="J52" s="15" t="inlineStr"/>
+      <c r="K52" s="15" t="inlineStr"/>
+      <c r="L52" s="15" t="inlineStr"/>
+      <c r="M52" s="15" t="inlineStr"/>
+      <c r="N52" s="15" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="16" t="n">
@@ -3700,12 +3702,12 @@
       </c>
       <c r="B53" s="16" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C53" s="16" t="inlineStr">
         <is>
-          <t>Final reconciliation report</t>
+          <t>Agree the hypercare window before you need it</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
@@ -3715,7 +3717,7 @@
       </c>
       <c r="E53" s="16" t="inlineStr">
         <is>
-          <t>Migration Lead</t>
+          <t>Client PM</t>
         </is>
       </c>
       <c r="F53" s="16" t="inlineStr">
@@ -3729,14 +3731,12 @@
       <c r="H53" s="16" t="n"/>
       <c r="I53" s="16" t="n"/>
       <c r="J53" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="K53" s="16" t="n">
-        <v>43</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K53" s="16" t="inlineStr"/>
       <c r="L53" s="16" t="inlineStr">
         <is>
-          <t>The proof the move was complete</t>
+          <t>Length and route agreed in advance</t>
         </is>
       </c>
       <c r="M53" s="16" t="inlineStr">
@@ -3752,12 +3752,12 @@
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="C54" s="16" t="inlineStr">
         <is>
-          <t>Internal results readout</t>
+          <t>Log and resolve what surfaces</t>
         </is>
       </c>
       <c r="D54" s="16" t="inlineStr">
@@ -3781,14 +3781,14 @@
       <c r="H54" s="16" t="n"/>
       <c r="I54" s="16" t="n"/>
       <c r="J54" s="16" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="K54" s="16" t="n">
         <v>44</v>
       </c>
       <c r="L54" s="16" t="inlineStr">
         <is>
-          <t>What went well, what to change next time</t>
+          <t>The long tail, tracked not absorbed</t>
         </is>
       </c>
       <c r="M54" s="16" t="inlineStr">
@@ -3804,12 +3804,12 @@
       </c>
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="C55" s="16" t="inlineStr">
         <is>
-          <t>Handoff to Support</t>
+          <t>Final reconciliation report</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
@@ -3819,7 +3819,7 @@
       </c>
       <c r="E55" s="16" t="inlineStr">
         <is>
-          <t>Support / CS</t>
+          <t>Migration Lead</t>
         </is>
       </c>
       <c r="F55" s="16" t="inlineStr">
@@ -3833,200 +3833,202 @@
       <c r="H55" s="16" t="n"/>
       <c r="I55" s="16" t="n"/>
       <c r="J55" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K55" s="16" t="n">
         <v>45</v>
       </c>
       <c r="L55" s="16" t="inlineStr">
         <is>
+          <t>The proof the move was complete</t>
+        </is>
+      </c>
+      <c r="M55" s="16" t="inlineStr">
+        <is>
+          <t>migration-hypercare</t>
+        </is>
+      </c>
+      <c r="N55" s="16" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="16" t="n">
+        <v>47</v>
+      </c>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>8.4</t>
+        </is>
+      </c>
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>Internal results readout</t>
+        </is>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>Stage 8 — Hypercare and Close</t>
+        </is>
+      </c>
+      <c r="E56" s="16" t="inlineStr">
+        <is>
+          <t>Migration Lead</t>
+        </is>
+      </c>
+      <c r="F56" s="16" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G56" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="16" t="n"/>
+      <c r="I56" s="16" t="n"/>
+      <c r="J56" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K56" s="16" t="n">
+        <v>46</v>
+      </c>
+      <c r="L56" s="16" t="inlineStr">
+        <is>
+          <t>What went well, what to change next time</t>
+        </is>
+      </c>
+      <c r="M56" s="16" t="inlineStr">
+        <is>
+          <t>migration-hypercare</t>
+        </is>
+      </c>
+      <c r="N56" s="16" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="n">
+        <v>48</v>
+      </c>
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>Handoff to Support</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Stage 8 — Hypercare and Close</t>
+        </is>
+      </c>
+      <c r="E57" s="16" t="inlineStr">
+        <is>
+          <t>Support / CS</t>
+        </is>
+      </c>
+      <c r="F57" s="16" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G57" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="16" t="n"/>
+      <c r="I57" s="16" t="n"/>
+      <c r="J57" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="K57" s="16" t="n">
+        <v>47</v>
+      </c>
+      <c r="L57" s="16" t="inlineStr">
+        <is>
           <t>So it lands warmly, with context</t>
         </is>
       </c>
-      <c r="M55" s="16" t="inlineStr">
+      <c r="M57" s="16" t="inlineStr">
         <is>
           <t>migration-hypercare</t>
         </is>
       </c>
-      <c r="N55" s="16" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="18" t="n">
-        <v>47</v>
-      </c>
-      <c r="B56" s="18" t="inlineStr">
+      <c r="N57" s="16" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="18" t="n">
+        <v>49</v>
+      </c>
+      <c r="B58" s="18" t="inlineStr">
         <is>
           <t>8.6</t>
         </is>
       </c>
-      <c r="C56" s="19" t="inlineStr">
+      <c r="C58" s="19" t="inlineStr">
         <is>
           <t>GATE — project closed, handoff accepted</t>
         </is>
       </c>
-      <c r="D56" s="18" t="inlineStr">
+      <c r="D58" s="18" t="inlineStr">
         <is>
           <t>Stage 8 — Hypercare and Close</t>
         </is>
       </c>
-      <c r="E56" s="18" t="inlineStr">
+      <c r="E58" s="18" t="inlineStr">
         <is>
           <t>Support / CS</t>
         </is>
       </c>
-      <c r="F56" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G56" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="18" t="n"/>
-      <c r="I56" s="18" t="n"/>
-      <c r="J56" s="18" t="n">
+      <c r="F58" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G58" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="18" t="n"/>
+      <c r="I58" s="18" t="n"/>
+      <c r="J58" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="K56" s="18" t="n">
-        <v>46</v>
-      </c>
-      <c r="L56" s="18" t="inlineStr">
+      <c r="K58" s="18" t="n">
+        <v>48</v>
+      </c>
+      <c r="L58" s="18" t="inlineStr">
         <is>
           <t>Support owns it now, knowingly</t>
         </is>
       </c>
-      <c r="M56" s="18" t="inlineStr">
+      <c r="M58" s="18" t="inlineStr">
         <is>
           <t>migration-hypercare</t>
         </is>
       </c>
-      <c r="N56" s="18" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="15" t="inlineStr"/>
-      <c r="B57" s="15" t="inlineStr">
+      <c r="N58" s="18" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr"/>
+      <c r="B59" s="15" t="inlineStr">
         <is>
           <t>DD</t>
         </is>
       </c>
-      <c r="C57" s="15" t="inlineStr">
+      <c r="C59" s="15" t="inlineStr">
         <is>
           <t>Parallel — Document Digitization</t>
         </is>
       </c>
-      <c r="D57" s="15" t="inlineStr"/>
-      <c r="E57" s="15" t="inlineStr"/>
-      <c r="F57" s="15" t="inlineStr"/>
-      <c r="G57" s="15" t="inlineStr"/>
-      <c r="H57" s="15" t="inlineStr"/>
-      <c r="I57" s="15" t="inlineStr"/>
-      <c r="J57" s="15" t="inlineStr"/>
-      <c r="K57" s="15" t="inlineStr"/>
-      <c r="L57" s="15" t="inlineStr"/>
-      <c r="M57" s="15" t="inlineStr"/>
-      <c r="N57" s="15" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="16" t="n">
-        <v>48</v>
-      </c>
-      <c r="B58" s="16" t="inlineStr">
-        <is>
-          <t>DD.1</t>
-        </is>
-      </c>
-      <c r="C58" s="16" t="inlineStr">
-        <is>
-          <t>Audit paper volume, condition and scope</t>
-        </is>
-      </c>
-      <c r="D58" s="16" t="inlineStr">
-        <is>
-          <t>Parallel — Document Digitization</t>
-        </is>
-      </c>
-      <c r="E58" s="16" t="inlineStr">
-        <is>
-          <t>Client Data Owner</t>
-        </is>
-      </c>
-      <c r="F58" s="16" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G58" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" s="16" t="n"/>
-      <c r="I58" s="16" t="n"/>
-      <c r="J58" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="K58" s="16" t="inlineStr"/>
-      <c r="L58" s="16" t="inlineStr">
-        <is>
-          <t>How much paper, in what state</t>
-        </is>
-      </c>
-      <c r="M58" s="16" t="inlineStr">
-        <is>
-          <t>migration-field-mapping</t>
-        </is>
-      </c>
-      <c r="N58" s="16" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="16" t="n">
-        <v>49</v>
-      </c>
-      <c r="B59" s="16" t="inlineStr">
-        <is>
-          <t>DD.2</t>
-        </is>
-      </c>
-      <c r="C59" s="16" t="inlineStr">
-        <is>
-          <t>Select vendor and agree chain of custody</t>
-        </is>
-      </c>
-      <c r="D59" s="16" t="inlineStr">
-        <is>
-          <t>Parallel — Document Digitization</t>
-        </is>
-      </c>
-      <c r="E59" s="16" t="inlineStr">
-        <is>
-          <t>Client PM</t>
-        </is>
-      </c>
-      <c r="F59" s="16" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G59" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H59" s="16" t="n"/>
-      <c r="I59" s="16" t="n"/>
-      <c r="J59" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="K59" s="16" t="n">
-        <v>48</v>
-      </c>
-      <c r="L59" s="16" t="inlineStr">
-        <is>
-          <t>Who holds the records, and how it is proven</t>
-        </is>
-      </c>
-      <c r="M59" s="16" t="inlineStr">
-        <is>
-          <t>migration-field-mapping</t>
-        </is>
-      </c>
-      <c r="N59" s="16" t="inlineStr"/>
+      <c r="D59" s="15" t="inlineStr"/>
+      <c r="E59" s="15" t="inlineStr"/>
+      <c r="F59" s="15" t="inlineStr"/>
+      <c r="G59" s="15" t="inlineStr"/>
+      <c r="H59" s="15" t="inlineStr"/>
+      <c r="I59" s="15" t="inlineStr"/>
+      <c r="J59" s="15" t="inlineStr"/>
+      <c r="K59" s="15" t="inlineStr"/>
+      <c r="L59" s="15" t="inlineStr"/>
+      <c r="M59" s="15" t="inlineStr"/>
+      <c r="N59" s="15" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="16" t="n">
@@ -4034,12 +4036,12 @@
       </c>
       <c r="B60" s="16" t="inlineStr">
         <is>
-          <t>DD.3</t>
+          <t>DD.1</t>
         </is>
       </c>
       <c r="C60" s="16" t="inlineStr">
         <is>
-          <t>Define indexing metadata to match the map</t>
+          <t>Audit paper volume, condition and scope</t>
         </is>
       </c>
       <c r="D60" s="16" t="inlineStr">
@@ -4049,7 +4051,7 @@
       </c>
       <c r="E60" s="16" t="inlineStr">
         <is>
-          <t>Migration Lead</t>
+          <t>Client Data Owner</t>
         </is>
       </c>
       <c r="F60" s="16" t="inlineStr">
@@ -4063,14 +4065,12 @@
       <c r="H60" s="16" t="n"/>
       <c r="I60" s="16" t="n"/>
       <c r="J60" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="K60" s="16" t="n">
-        <v>49</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="K60" s="16" t="inlineStr"/>
       <c r="L60" s="16" t="inlineStr">
         <is>
-          <t>Index to the target fields, not to what is convenient</t>
+          <t>How much paper, in what state</t>
         </is>
       </c>
       <c r="M60" s="16" t="inlineStr">
@@ -4086,12 +4086,12 @@
       </c>
       <c r="B61" s="16" t="inlineStr">
         <is>
-          <t>DD.4</t>
+          <t>DD.2</t>
         </is>
       </c>
       <c r="C61" s="16" t="inlineStr">
         <is>
-          <t>Scan, OCR, index and QA</t>
+          <t>Select vendor and agree chain of custody</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="E61" s="16" t="inlineStr">
         <is>
-          <t>Scanning Vendor</t>
+          <t>Client PM</t>
         </is>
       </c>
       <c r="F61" s="16" t="inlineStr">
@@ -4115,14 +4115,14 @@
       <c r="H61" s="16" t="n"/>
       <c r="I61" s="16" t="n"/>
       <c r="J61" s="16" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="K61" s="16" t="n">
         <v>50</v>
       </c>
       <c r="L61" s="16" t="inlineStr">
         <is>
-          <t>Digitized and indexed, ready to link</t>
+          <t>Who holds the records, and how it is proven</t>
         </is>
       </c>
       <c r="M61" s="16" t="inlineStr">
@@ -4138,12 +4138,12 @@
       </c>
       <c r="B62" s="16" t="inlineStr">
         <is>
-          <t>DD.5</t>
+          <t>DD.3</t>
         </is>
       </c>
       <c r="C62" s="16" t="inlineStr">
         <is>
-          <t>Day-forward scanning live at go-live</t>
+          <t>Define indexing metadata to match the map</t>
         </is>
       </c>
       <c r="D62" s="16" t="inlineStr">
@@ -4153,7 +4153,7 @@
       </c>
       <c r="E62" s="16" t="inlineStr">
         <is>
-          <t>Scanning Vendor</t>
+          <t>Migration Lead</t>
         </is>
       </c>
       <c r="F62" s="16" t="inlineStr">
@@ -4167,64 +4167,92 @@
       <c r="H62" s="16" t="n"/>
       <c r="I62" s="16" t="n"/>
       <c r="J62" s="16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K62" s="16" t="n">
         <v>51</v>
       </c>
       <c r="L62" s="16" t="inlineStr">
         <is>
-          <t>New paper never becomes new backlog</t>
+          <t>Index to the target fields, not to what is convenient</t>
         </is>
       </c>
       <c r="M62" s="16" t="inlineStr">
         <is>
-          <t>migration-cutover</t>
+          <t>migration-field-mapping</t>
         </is>
       </c>
       <c r="N62" s="16" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="15" t="inlineStr"/>
-      <c r="B63" s="15" t="inlineStr">
-        <is>
-          <t>BF</t>
-        </is>
-      </c>
-      <c r="C63" s="15" t="inlineStr">
-        <is>
-          <t>Follow-on — Backfile (T plus 6 months)</t>
-        </is>
-      </c>
-      <c r="D63" s="15" t="inlineStr"/>
-      <c r="E63" s="15" t="inlineStr"/>
-      <c r="F63" s="15" t="inlineStr"/>
-      <c r="G63" s="15" t="inlineStr"/>
-      <c r="H63" s="15" t="inlineStr"/>
-      <c r="I63" s="15" t="inlineStr"/>
-      <c r="J63" s="15" t="inlineStr"/>
-      <c r="K63" s="15" t="inlineStr"/>
-      <c r="L63" s="15" t="inlineStr"/>
-      <c r="M63" s="15" t="inlineStr"/>
-      <c r="N63" s="15" t="inlineStr"/>
+      <c r="A63" s="16" t="n">
+        <v>53</v>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>DD.4</t>
+        </is>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>Scan, OCR, index and QA</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>Parallel — Document Digitization</t>
+        </is>
+      </c>
+      <c r="E63" s="16" t="inlineStr">
+        <is>
+          <t>Scanning Vendor</t>
+        </is>
+      </c>
+      <c r="F63" s="16" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G63" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" s="16" t="n"/>
+      <c r="I63" s="16" t="n"/>
+      <c r="J63" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="K63" s="16" t="n">
+        <v>52</v>
+      </c>
+      <c r="L63" s="16" t="inlineStr">
+        <is>
+          <t>Digitized and indexed, ready to link</t>
+        </is>
+      </c>
+      <c r="M63" s="16" t="inlineStr">
+        <is>
+          <t>migration-field-mapping</t>
+        </is>
+      </c>
+      <c r="N63" s="16" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="16" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B64" s="16" t="inlineStr">
         <is>
-          <t>BF.1</t>
+          <t>DD.5</t>
         </is>
       </c>
       <c r="C64" s="16" t="inlineStr">
         <is>
-          <t>Backfile scanning continues</t>
+          <t>Day-forward scanning live at go-live</t>
         </is>
       </c>
       <c r="D64" s="16" t="inlineStr">
         <is>
-          <t>Follow-on — Backfile (T plus 6 months)</t>
+          <t>Parallel — Document Digitization</t>
         </is>
       </c>
       <c r="E64" s="16" t="inlineStr">
@@ -4243,72 +4271,46 @@
       <c r="H64" s="16" t="n"/>
       <c r="I64" s="16" t="n"/>
       <c r="J64" s="16" t="n">
-        <v>90</v>
-      </c>
-      <c r="K64" s="16" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K64" s="16" t="n">
+        <v>53</v>
+      </c>
       <c r="L64" s="16" t="inlineStr">
         <is>
-          <t>The historical paper, on contract</t>
+          <t>New paper never becomes new backlog</t>
         </is>
       </c>
       <c r="M64" s="16" t="inlineStr">
         <is>
-          <t>migration-hypercare</t>
+          <t>migration-cutover</t>
         </is>
       </c>
       <c r="N64" s="16" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="16" t="n">
-        <v>54</v>
-      </c>
-      <c r="B65" s="16" t="inlineStr">
-        <is>
-          <t>BF.2</t>
-        </is>
-      </c>
-      <c r="C65" s="16" t="inlineStr">
-        <is>
-          <t>Bridge import of historical documents</t>
-        </is>
-      </c>
-      <c r="D65" s="16" t="inlineStr">
+      <c r="A65" s="15" t="inlineStr"/>
+      <c r="B65" s="15" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="C65" s="15" t="inlineStr">
         <is>
           <t>Follow-on — Backfile (T plus 6 months)</t>
         </is>
       </c>
-      <c r="E65" s="16" t="inlineStr">
-        <is>
-          <t>Migration Lead</t>
-        </is>
-      </c>
-      <c r="F65" s="16" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G65" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H65" s="16" t="n"/>
-      <c r="I65" s="16" t="n"/>
-      <c r="J65" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="K65" s="16" t="n">
-        <v>53</v>
-      </c>
-      <c r="L65" s="16" t="inlineStr">
-        <is>
-          <t>Loaded and linked by the same unique ID</t>
-        </is>
-      </c>
-      <c r="M65" s="16" t="inlineStr">
-        <is>
-          <t>migration-field-mapping</t>
-        </is>
-      </c>
-      <c r="N65" s="16" t="inlineStr"/>
+      <c r="D65" s="15" t="inlineStr"/>
+      <c r="E65" s="15" t="inlineStr"/>
+      <c r="F65" s="15" t="inlineStr"/>
+      <c r="G65" s="15" t="inlineStr"/>
+      <c r="H65" s="15" t="inlineStr"/>
+      <c r="I65" s="15" t="inlineStr"/>
+      <c r="J65" s="15" t="inlineStr"/>
+      <c r="K65" s="15" t="inlineStr"/>
+      <c r="L65" s="15" t="inlineStr"/>
+      <c r="M65" s="15" t="inlineStr"/>
+      <c r="N65" s="15" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="16" t="n">
@@ -4316,12 +4318,12 @@
       </c>
       <c r="B66" s="16" t="inlineStr">
         <is>
-          <t>BF.3</t>
+          <t>BF.1</t>
         </is>
       </c>
       <c r="C66" s="16" t="inlineStr">
         <is>
-          <t>Reconcile the backfile</t>
+          <t>Backfile scanning continues</t>
         </is>
       </c>
       <c r="D66" s="16" t="inlineStr">
@@ -4331,7 +4333,7 @@
       </c>
       <c r="E66" s="16" t="inlineStr">
         <is>
-          <t>Migration Lead</t>
+          <t>Scanning Vendor</t>
         </is>
       </c>
       <c r="F66" s="16" t="inlineStr">
@@ -4345,19 +4347,17 @@
       <c r="H66" s="16" t="n"/>
       <c r="I66" s="16" t="n"/>
       <c r="J66" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="K66" s="16" t="n">
-        <v>54</v>
-      </c>
+        <v>90</v>
+      </c>
+      <c r="K66" s="16" t="inlineStr"/>
       <c r="L66" s="16" t="inlineStr">
         <is>
-          <t>Counts tie, no orphans</t>
+          <t>The historical paper, on contract</t>
         </is>
       </c>
       <c r="M66" s="16" t="inlineStr">
         <is>
-          <t>migration-pitfalls</t>
+          <t>migration-hypercare</t>
         </is>
       </c>
       <c r="N66" s="16" t="inlineStr"/>
@@ -4368,12 +4368,12 @@
       </c>
       <c r="B67" s="16" t="inlineStr">
         <is>
-          <t>BF.4</t>
+          <t>BF.2</t>
         </is>
       </c>
       <c r="C67" s="16" t="inlineStr">
         <is>
-          <t>Decommission paper storage</t>
+          <t>Bridge import of historical documents</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="E67" s="16" t="inlineStr">
         <is>
-          <t>Client PM</t>
+          <t>Migration Lead</t>
         </is>
       </c>
       <c r="F67" s="16" t="inlineStr">
@@ -4404,19 +4404,123 @@
       </c>
       <c r="L67" s="16" t="inlineStr">
         <is>
+          <t>Loaded and linked by the same unique ID</t>
+        </is>
+      </c>
+      <c r="M67" s="16" t="inlineStr">
+        <is>
+          <t>migration-field-mapping</t>
+        </is>
+      </c>
+      <c r="N67" s="16" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="16" t="n">
+        <v>57</v>
+      </c>
+      <c r="B68" s="16" t="inlineStr">
+        <is>
+          <t>BF.3</t>
+        </is>
+      </c>
+      <c r="C68" s="16" t="inlineStr">
+        <is>
+          <t>Reconcile the backfile</t>
+        </is>
+      </c>
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>Follow-on — Backfile (T plus 6 months)</t>
+        </is>
+      </c>
+      <c r="E68" s="16" t="inlineStr">
+        <is>
+          <t>Migration Lead</t>
+        </is>
+      </c>
+      <c r="F68" s="16" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G68" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="16" t="n"/>
+      <c r="I68" s="16" t="n"/>
+      <c r="J68" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="K68" s="16" t="n">
+        <v>56</v>
+      </c>
+      <c r="L68" s="16" t="inlineStr">
+        <is>
+          <t>Counts tie, no orphans</t>
+        </is>
+      </c>
+      <c r="M68" s="16" t="inlineStr">
+        <is>
+          <t>migration-pitfalls</t>
+        </is>
+      </c>
+      <c r="N68" s="16" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="16" t="n">
+        <v>58</v>
+      </c>
+      <c r="B69" s="16" t="inlineStr">
+        <is>
+          <t>BF.4</t>
+        </is>
+      </c>
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>Decommission paper storage</t>
+        </is>
+      </c>
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>Follow-on — Backfile (T plus 6 months)</t>
+        </is>
+      </c>
+      <c r="E69" s="16" t="inlineStr">
+        <is>
+          <t>Client PM</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G69" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" s="16" t="n"/>
+      <c r="I69" s="16" t="n"/>
+      <c r="J69" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="K69" s="16" t="n">
+        <v>57</v>
+      </c>
+      <c r="L69" s="16" t="inlineStr">
+        <is>
           <t>The reason the project was funded</t>
         </is>
       </c>
-      <c r="M67" s="16" t="inlineStr">
+      <c r="M69" s="16" t="inlineStr">
         <is>
           <t>migration-hypercare</t>
         </is>
       </c>
-      <c r="N67" s="16" t="inlineStr"/>
+      <c r="N69" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,In Progress,Done,Blocked,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4498,7 +4602,7 @@
         </is>
       </c>
       <c r="B2" s="22" t="n">
-        <v>46097</v>
+        <v>46090</v>
       </c>
       <c r="C2" s="21" t="inlineStr">
         <is>
@@ -4526,7 +4630,7 @@
         </is>
       </c>
       <c r="H2" s="22" t="n">
-        <v>46099</v>
+        <v>46092</v>
       </c>
       <c r="I2" s="21" t="inlineStr"/>
     </row>
@@ -4627,7 +4731,7 @@
         </is>
       </c>
       <c r="B2" s="22" t="n">
-        <v>46086</v>
+        <v>46079</v>
       </c>
       <c r="C2" s="21" t="inlineStr">
         <is>
@@ -4665,7 +4769,7 @@
         </is>
       </c>
       <c r="J2" s="22" t="n">
-        <v>46090</v>
+        <v>46083</v>
       </c>
     </row>
     <row r="4">
@@ -4783,7 +4887,7 @@
         </is>
       </c>
       <c r="H2" s="22" t="n">
-        <v>46150</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="4">

</xml_diff>